<commit_message>
Update the SaaS plan details and export to Excel
Update the Excel export to include customization pricing and update the metadata title.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: e70c97c4-e099-455a-b9ae-aa9a0dedb718
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 76e33437-a5bb-4543-9f00-23c5d1e762de
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/713657ac-53c6-43a9-97a8-ef2697ef92d9/e70c97c4-e099-455a-b9ae-aa9a0dedb718/Ho5yVHe
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/Kinto_SaaS_Multitenancy_Plan.xlsx
+++ b/Kinto_SaaS_Multitenancy_Plan.xlsx
@@ -11,13 +11,14 @@
     <sheet sheetId="5" name="Implementation Phases" state="visible" r:id="rId8"/>
     <sheet sheetId="6" name="SaaS &amp; Deployment" state="visible" r:id="rId9"/>
     <sheet sheetId="7" name="Integrations Impact" state="visible" r:id="rId10"/>
+    <sheet sheetId="8" name="Customization Pricing" state="visible" r:id="rId11"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="529" uniqueCount="348">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="584" uniqueCount="398">
   <si>
     <t>KINTO SMART OPS — MULTITENANCY &amp; SAAS PLAN</t>
   </si>
@@ -673,7 +674,7 @@
     <t>Grace period begins. Read-only mode.</t>
   </si>
   <si>
-    <t>Day 1-7</t>
+    <t>Day 1–7</t>
   </si>
   <si>
     <t>User can view all data but cannot create new records. Reminder emails sent.</t>
@@ -685,7 +686,7 @@
     <t>Account suspended. Login blocked. Data fully preserved.</t>
   </si>
   <si>
-    <t>Day 8-90</t>
+    <t>Day 8–90</t>
   </si>
   <si>
     <t>Data retained. Reactivate anytime by renewing subscription.</t>
@@ -721,7 +722,7 @@
     <t>Days</t>
   </si>
   <si>
-    <t>Cumulative</t>
+    <t>Cumul.</t>
   </si>
   <si>
     <t>Priority</t>
@@ -808,7 +809,7 @@
     <t>Cross-tenant data leak tests. Module enforcement tests. Billing flow tests. Load testing. Security audit. UAT with KINTO.</t>
   </si>
   <si>
-    <t>TOTAL ESTIMATED EFFORT: ~33–36 working days  |  ~7–8 weeks  |  Timeline depends on parallel development capacity</t>
+    <t>TOTAL ESTIMATED EFFORT: ~33–36 working days  |  ~7–8 weeks</t>
   </si>
   <si>
     <t>WHAT STAYS EXACTLY THE SAME (ZERO CHANGES)</t>
@@ -868,7 +869,7 @@
     <t>AWS EC2 + RDS (Mumbai region)</t>
   </si>
   <si>
-    <t>More control. Indian data residency. Cost-effective at scale. No code change except file storage.</t>
+    <t>More control. Indian data residency. Cost-effective at scale.</t>
   </si>
   <si>
     <t>₹8,000–20,000/mo</t>
@@ -907,72 +908,60 @@
     <t>No EC2, no Docker, no Linux, no DevOps needed</t>
   </si>
   <si>
-    <t>CODE CHANGES NEEDED FOR CLOUD (AWS/GCP) — only if moving beyond Replit</t>
-  </si>
-  <si>
-    <t>Component</t>
-  </si>
-  <si>
-    <t>Change Required</t>
-  </si>
-  <si>
-    <t>Easy</t>
+    <t>SAAS BUSINESS MODEL</t>
+  </si>
+  <si>
+    <t>Item</t>
+  </si>
+  <si>
+    <t>= SaaS Vendor. Your company uses the system for free as Tenant 1.</t>
+  </si>
+  <si>
+    <t>= Manufacturing companies paying monthly subscriptions.</t>
+  </si>
+  <si>
+    <t>MRR (Monthly Recurring Revenue) from all active tenants.</t>
+  </si>
+  <si>
+    <t>Customers sign up, complete wizard, start 14-day trial, choose plan, pay via Razorpay.</t>
+  </si>
+  <si>
+    <t>Starter → Professional → Enterprise as companies grow.</t>
+  </si>
+  <si>
+    <t>Razorpay supports UPI, NEFT, credit/debit cards — best for Indian B2B.</t>
+  </si>
+  <si>
+    <t>Offer 2 months free on annual plan to encourage commitment.</t>
+  </si>
+  <si>
+    <t>50 tenants or 500 tenants — same codebase, same Replit deployment until you need more.</t>
+  </si>
+  <si>
+    <t>INTEGRATIONS &amp; SERVICES IMPACT</t>
+  </si>
+  <si>
+    <t>WhatsApp  |  Email  |  Files  |  Reports  |  API</t>
+  </si>
+  <si>
+    <t>WHATSAPP INTEGRATION</t>
+  </si>
+  <si>
+    <t>Aspect</t>
+  </si>
+  <si>
+    <t>Current</t>
+  </si>
+  <si>
+    <t>After Multitenancy</t>
+  </si>
+  <si>
+    <t>Credentials</t>
   </si>
   <si>
     <t>Low</t>
   </si>
   <si>
-    <t>SAAS BUSINESS MODEL</t>
-  </si>
-  <si>
-    <t>Item</t>
-  </si>
-  <si>
-    <t>= SaaS Vendor. Your company uses the system for free as Tenant 1.</t>
-  </si>
-  <si>
-    <t>= Manufacturing companies paying monthly subscriptions.</t>
-  </si>
-  <si>
-    <t>MRR (Monthly Recurring Revenue) from all active tenants.</t>
-  </si>
-  <si>
-    <t>Customers sign up, complete wizard, start 14-day trial, choose plan, pay via Razorpay.</t>
-  </si>
-  <si>
-    <t>Starter → Professional → Enterprise as companies grow.</t>
-  </si>
-  <si>
-    <t>Razorpay supports UPI, NEFT, credit/debit cards — best for Indian B2B.</t>
-  </si>
-  <si>
-    <t>Offer 2 months free on annual plan to encourage commitment.</t>
-  </si>
-  <si>
-    <t>50 tenants or 500 tenants — same codebase, same Replit deployment until you need more.</t>
-  </si>
-  <si>
-    <t>INTEGRATIONS &amp; SERVICES IMPACT</t>
-  </si>
-  <si>
-    <t>WhatsApp  |  Email  |  Files  |  Reports  |  API</t>
-  </si>
-  <si>
-    <t>WHATSAPP INTEGRATION</t>
-  </si>
-  <si>
-    <t>Aspect</t>
-  </si>
-  <si>
-    <t>Current</t>
-  </si>
-  <si>
-    <t>After Multitenancy</t>
-  </si>
-  <si>
-    <t>Credentials</t>
-  </si>
-  <si>
     <t>Incoming webhook</t>
   </si>
   <si>
@@ -982,36 +971,27 @@
     <t>Checklist completion</t>
   </si>
   <si>
-    <t>Tenant without own number</t>
+    <t>EMAIL NOTIFICATIONS</t>
+  </si>
+  <si>
+    <t>Setting</t>
+  </si>
+  <si>
+    <t>Sender name</t>
+  </si>
+  <si>
+    <t>Reply-to</t>
+  </si>
+  <si>
+    <t>Email logo</t>
+  </si>
+  <si>
+    <t>Machine reminders</t>
   </si>
   <si>
     <t>None</t>
   </si>
   <si>
-    <t>EMAIL NOTIFICATIONS</t>
-  </si>
-  <si>
-    <t>Setting</t>
-  </si>
-  <si>
-    <t>Sender name</t>
-  </si>
-  <si>
-    <t>Reply-to</t>
-  </si>
-  <si>
-    <t>Email logo</t>
-  </si>
-  <si>
-    <t>Machine startup reminders</t>
-  </si>
-  <si>
-    <t>None (auto via tenant_id)</t>
-  </si>
-  <si>
-    <t>Missed checklist alerts</t>
-  </si>
-  <si>
     <t>Document expiry alerts</t>
   </si>
   <si>
@@ -1042,6 +1022,9 @@
     <t>Report</t>
   </si>
   <si>
+    <t>Change</t>
+  </si>
+  <si>
     <t>All operational reports</t>
   </si>
   <si>
@@ -1060,14 +1043,182 @@
     <t>Super Admin MRR report</t>
   </si>
   <si>
-    <t>Super Admin storage report</t>
+    <t>CUSTOMIZATION PRICING</t>
+  </si>
+  <si>
+    <t>Fixed Price Model  |  One Clear Rate  |  No Hourly Billing</t>
+  </si>
+  <si>
+    <t>RULE: All customizations are Fixed Price only. Quote upfront. Customer approves before work starts. No hourly billing. No ambiguity.</t>
+  </si>
+  <si>
+    <t>CUSTOMIZATION PRICE LIST</t>
+  </si>
+  <si>
+    <t>Customization Type</t>
+  </si>
+  <si>
+    <t>Min Price</t>
+  </si>
+  <si>
+    <t>Max Price</t>
+  </si>
+  <si>
+    <t>What It Includes</t>
+  </si>
+  <si>
+    <t>Custom Report</t>
+  </si>
+  <si>
+    <t>₹5,000</t>
+  </si>
+  <si>
+    <t>₹15,000</t>
+  </si>
+  <si>
+    <t>New Excel or PDF report specific to one customer — layout, data, columns as per their requirement</t>
+  </si>
+  <si>
+    <t>Custom Fields in a Module</t>
+  </si>
+  <si>
+    <t>₹3,000</t>
+  </si>
+  <si>
+    <t>₹8,000</t>
+  </si>
+  <si>
+    <t>Additional fields not in standard forms — invoices, production, checklist, etc.</t>
+  </si>
+  <si>
+    <t>Custom Workflow / Approval Flow</t>
+  </si>
+  <si>
+    <t>₹10,000</t>
+  </si>
+  <si>
+    <t>₹30,000</t>
+  </si>
+  <si>
+    <t>Different approval stages, state changes, rules or conditions specific to one customer</t>
+  </si>
+  <si>
+    <t>API / Tally / ERP Integration</t>
+  </si>
+  <si>
+    <t>₹50,000</t>
+  </si>
+  <si>
+    <t>Connect Kinto with customer's existing Tally, ERP, or third-party software via API</t>
+  </si>
+  <si>
+    <t>WhatsApp Custom Flow</t>
+  </si>
+  <si>
+    <t>₹20,000</t>
+  </si>
+  <si>
+    <t>Custom bot messages, custom checklist templates, custom reminder logic for WhatsApp</t>
+  </si>
+  <si>
+    <t>Custom MIS Dashboard</t>
+  </si>
+  <si>
+    <t>₹25,000</t>
+  </si>
+  <si>
+    <t>New MIS widgets, KPIs, charts or analytics screens specific to customer's operations</t>
+  </si>
+  <si>
+    <t>Data Migration (Historical Import)</t>
+  </si>
+  <si>
+    <t>Import customer's historical data from Excel, Tally, or other software into Kinto</t>
+  </si>
+  <si>
+    <t>Training Session</t>
+  </si>
+  <si>
+    <t>Per session — on-site or remote training for customer's team (per session rate)</t>
+  </si>
+  <si>
+    <t>Priority Support SLA (Monthly)</t>
+  </si>
+  <si>
+    <t>₹2,000/mo</t>
+  </si>
+  <si>
+    <t>₹5,000/mo</t>
+  </si>
+  <si>
+    <t>Guaranteed response time add-on (e.g. 4-hour response). Billed monthly on top of subscription.</t>
+  </si>
+  <si>
+    <t>THE PROCESS — HOW EVERY CUSTOMIZATION WORKS</t>
+  </si>
+  <si>
+    <t>Action</t>
+  </si>
+  <si>
+    <t>Who Does It</t>
+  </si>
+  <si>
+    <t>Customer</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>Kinto team</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>Both</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>WHAT IS INCLUDED IN SUBSCRIPTION (NO EXTRA CHARGE)</t>
+  </si>
+  <si>
+    <t>Standard features available to all tenants on their plan</t>
+  </si>
+  <si>
+    <t>Bug fixes and error corrections in existing functionality</t>
+  </si>
+  <si>
+    <t>New platform features released by Kinto to all tenants (everyone gets them automatically)</t>
+  </si>
+  <si>
+    <t>Configuration within the app — roles, permissions, categories, expense types, chart of accounts, etc.</t>
+  </si>
+  <si>
+    <t>Email and WhatsApp support for how-to questions within standard usage</t>
+  </si>
+  <si>
+    <t>KEY RULE: STANDARD vs CUSTOM</t>
+  </si>
+  <si>
+    <t>If a customization built for one customer is useful to all customers → add it to the standard platform (free for everyone, grows the product). If it is specific only to that one customer → charge separately and maintain it as their private feature.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -1141,6 +1292,17 @@
     <font>
       <b/>
       <color rgb="FF1E293B"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF14532D"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <color rgb="FF78350F"/>
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
@@ -1251,7 +1413,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1358,6 +1520,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3986,7 +4157,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G36"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -4222,31 +4393,33 @@
       <c r="F19" s="3"/>
       <c r="G19" s="3"/>
     </row>
-    <row r="20" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="7" t="s">
         <v>297</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>298</v>
+        <v>10</v>
       </c>
       <c r="C20" s="7"/>
       <c r="D20" s="7"/>
       <c r="E20" s="7"/>
       <c r="F20" s="7"/>
-    </row>
-    <row r="21" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G20" s="7"/>
+    </row>
+    <row r="21" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
         <v>91</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>247</v>
+        <v>298</v>
       </c>
       <c r="C21" s="4"/>
       <c r="D21" s="4"/>
       <c r="E21" s="4"/>
       <c r="F21" s="4"/>
-    </row>
-    <row r="22" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G21" s="4"/>
+    </row>
+    <row r="22" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="8" t="s">
         <v>91</v>
       </c>
@@ -4257,173 +4430,88 @@
       <c r="D22" s="8"/>
       <c r="E22" s="8"/>
       <c r="F22" s="8"/>
-    </row>
-    <row r="23" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G22" s="8"/>
+    </row>
+    <row r="23" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
         <v>91</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C23" s="4"/>
       <c r="D23" s="4"/>
       <c r="E23" s="4"/>
       <c r="F23" s="4"/>
-    </row>
-    <row r="24" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G23" s="4"/>
+    </row>
+    <row r="24" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="8" t="s">
         <v>91</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C24" s="8"/>
       <c r="D24" s="8"/>
       <c r="E24" s="8"/>
       <c r="F24" s="8"/>
-    </row>
-    <row r="25" ht="18" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G24" s="8"/>
+    </row>
+    <row r="25" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
         <v>91</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="C25" s="4"/>
       <c r="D25" s="4"/>
       <c r="E25" s="4"/>
       <c r="F25" s="4"/>
-    </row>
-    <row r="27" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="3" t="s">
-        <v>301</v>
-      </c>
-      <c r="B27" s="3"/>
-      <c r="C27" s="3"/>
-      <c r="D27" s="3"/>
-      <c r="E27" s="3"/>
-      <c r="F27" s="3"/>
-      <c r="G27" s="3"/>
-    </row>
-    <row r="28" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="7" t="s">
-        <v>302</v>
-      </c>
-      <c r="B28" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="C28" s="7"/>
-      <c r="D28" s="7"/>
-      <c r="E28" s="7"/>
-      <c r="F28" s="7"/>
-      <c r="G28" s="7"/>
-    </row>
-    <row r="29" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="B29" s="4" t="s">
+      <c r="G25" s="4"/>
+    </row>
+    <row r="26" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="B26" s="8" t="s">
         <v>303</v>
       </c>
-      <c r="C29" s="4"/>
-      <c r="D29" s="4"/>
-      <c r="E29" s="4"/>
-      <c r="F29" s="4"/>
-      <c r="G29" s="4"/>
-    </row>
-    <row r="30" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="B30" s="8" t="s">
+      <c r="C26" s="8"/>
+      <c r="D26" s="8"/>
+      <c r="E26" s="8"/>
+      <c r="F26" s="8"/>
+      <c r="G26" s="8"/>
+    </row>
+    <row r="27" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B27" s="4" t="s">
         <v>304</v>
       </c>
-      <c r="C30" s="8"/>
-      <c r="D30" s="8"/>
-      <c r="E30" s="8"/>
-      <c r="F30" s="8"/>
-      <c r="G30" s="8"/>
-    </row>
-    <row r="31" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A31" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="B31" s="4" t="s">
+      <c r="C27" s="4"/>
+      <c r="D27" s="4"/>
+      <c r="E27" s="4"/>
+      <c r="F27" s="4"/>
+      <c r="G27" s="4"/>
+    </row>
+    <row r="28" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="B28" s="8" t="s">
         <v>305</v>
       </c>
-      <c r="C31" s="4"/>
-      <c r="D31" s="4"/>
-      <c r="E31" s="4"/>
-      <c r="F31" s="4"/>
-      <c r="G31" s="4"/>
-    </row>
-    <row r="32" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="B32" s="8" t="s">
-        <v>306</v>
-      </c>
-      <c r="C32" s="8"/>
-      <c r="D32" s="8"/>
-      <c r="E32" s="8"/>
-      <c r="F32" s="8"/>
-      <c r="G32" s="8"/>
-    </row>
-    <row r="33" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="B33" s="4" t="s">
-        <v>307</v>
-      </c>
-      <c r="C33" s="4"/>
-      <c r="D33" s="4"/>
-      <c r="E33" s="4"/>
-      <c r="F33" s="4"/>
-      <c r="G33" s="4"/>
-    </row>
-    <row r="34" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A34" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="B34" s="8" t="s">
-        <v>308</v>
-      </c>
-      <c r="C34" s="8"/>
-      <c r="D34" s="8"/>
-      <c r="E34" s="8"/>
-      <c r="F34" s="8"/>
-      <c r="G34" s="8"/>
-    </row>
-    <row r="35" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="B35" s="4" t="s">
-        <v>309</v>
-      </c>
-      <c r="C35" s="4"/>
-      <c r="D35" s="4"/>
-      <c r="E35" s="4"/>
-      <c r="F35" s="4"/>
-      <c r="G35" s="4"/>
-    </row>
-    <row r="36" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A36" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="B36" s="8" t="s">
-        <v>310</v>
-      </c>
-      <c r="C36" s="8"/>
-      <c r="D36" s="8"/>
-      <c r="E36" s="8"/>
-      <c r="F36" s="8"/>
-      <c r="G36" s="8"/>
+      <c r="C28" s="8"/>
+      <c r="D28" s="8"/>
+      <c r="E28" s="8"/>
+      <c r="F28" s="8"/>
+      <c r="G28" s="8"/>
     </row>
   </sheetData>
-  <mergeCells count="33">
+  <mergeCells count="26">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A3:G3"/>
@@ -4441,22 +4529,15 @@
     <mergeCell ref="B16:G16"/>
     <mergeCell ref="B17:G17"/>
     <mergeCell ref="A19:G19"/>
-    <mergeCell ref="B20:F20"/>
-    <mergeCell ref="B21:F21"/>
-    <mergeCell ref="B22:F22"/>
-    <mergeCell ref="B23:F23"/>
-    <mergeCell ref="B24:F24"/>
-    <mergeCell ref="B25:F25"/>
-    <mergeCell ref="A27:G27"/>
+    <mergeCell ref="B20:G20"/>
+    <mergeCell ref="B21:G21"/>
+    <mergeCell ref="B22:G22"/>
+    <mergeCell ref="B23:G23"/>
+    <mergeCell ref="B24:G24"/>
+    <mergeCell ref="B25:G25"/>
+    <mergeCell ref="B26:G26"/>
+    <mergeCell ref="B27:G27"/>
     <mergeCell ref="B28:G28"/>
-    <mergeCell ref="B29:G29"/>
-    <mergeCell ref="B30:G30"/>
-    <mergeCell ref="B31:G31"/>
-    <mergeCell ref="B32:G32"/>
-    <mergeCell ref="B33:G33"/>
-    <mergeCell ref="B34:G34"/>
-    <mergeCell ref="B35:G35"/>
-    <mergeCell ref="B36:G36"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -4465,7 +4546,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -4476,7 +4557,7 @@
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4487,7 +4568,7 @@
     </row>
     <row r="2" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>312</v>
+        <v>307</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -4498,7 +4579,7 @@
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
@@ -4509,13 +4590,13 @@
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
-        <v>314</v>
+        <v>309</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>316</v>
+        <v>311</v>
       </c>
       <c r="D4" s="7"/>
       <c r="E4" s="7"/>
@@ -4526,10 +4607,10 @@
         <v>91</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>317</v>
+        <v>312</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>300</v>
+        <v>313</v>
       </c>
       <c r="D5" s="4"/>
       <c r="E5" s="4"/>
@@ -4540,7 +4621,7 @@
         <v>91</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="C6" s="8" t="s">
         <v>256</v>
@@ -4554,10 +4635,10 @@
         <v>91</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>300</v>
+        <v>313</v>
       </c>
       <c r="D7" s="4"/>
       <c r="E7" s="4"/>
@@ -4568,186 +4649,186 @@
         <v>91</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>300</v>
+        <v>313</v>
       </c>
       <c r="D8" s="8"/>
       <c r="E8" s="8"/>
       <c r="F8" s="8"/>
     </row>
-    <row r="9" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="B9" s="4" t="s">
+    <row r="10" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>317</v>
+      </c>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+    </row>
+    <row r="11" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="7" t="s">
+        <v>318</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>310</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>311</v>
+      </c>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="7"/>
+    </row>
+    <row r="12" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>319</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>313</v>
+      </c>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
+      <c r="F12" s="4"/>
+    </row>
+    <row r="13" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>320</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>313</v>
+      </c>
+      <c r="D13" s="8"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="8"/>
+    </row>
+    <row r="14" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B14" s="4" t="s">
         <v>321</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C14" s="4" t="s">
+        <v>313</v>
+      </c>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4"/>
+      <c r="F14" s="4"/>
+    </row>
+    <row r="15" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="B15" s="8" t="s">
         <v>322</v>
       </c>
-      <c r="D9" s="4"/>
-      <c r="E9" s="4"/>
-      <c r="F9" s="4"/>
-    </row>
-    <row r="11" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
+      <c r="C15" s="8" t="s">
         <v>323</v>
       </c>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
-      <c r="G11" s="3"/>
-    </row>
-    <row r="12" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="7" t="s">
+      <c r="D15" s="8"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="8"/>
+    </row>
+    <row r="16" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B16" s="4" t="s">
         <v>324</v>
       </c>
-      <c r="B12" s="7" t="s">
-        <v>315</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>316</v>
-      </c>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
-    </row>
-    <row r="13" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="B13" s="4" t="s">
+      <c r="C16" s="4" t="s">
+        <v>323</v>
+      </c>
+      <c r="D16" s="4"/>
+      <c r="E16" s="4"/>
+      <c r="F16" s="4"/>
+    </row>
+    <row r="17" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="B17" s="8" t="s">
         <v>325</v>
       </c>
-      <c r="C13" s="4" t="s">
-        <v>300</v>
-      </c>
-      <c r="D13" s="4"/>
-      <c r="E13" s="4"/>
-      <c r="F13" s="4"/>
-    </row>
-    <row r="14" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="B14" s="8" t="s">
+      <c r="C17" s="8" t="s">
+        <v>256</v>
+      </c>
+      <c r="D17" s="8"/>
+      <c r="E17" s="8"/>
+      <c r="F17" s="8"/>
+    </row>
+    <row r="19" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
         <v>326</v>
       </c>
-      <c r="C14" s="8" t="s">
-        <v>300</v>
-      </c>
-      <c r="D14" s="8"/>
-      <c r="E14" s="8"/>
-      <c r="F14" s="8"/>
-    </row>
-    <row r="15" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="B15" s="4" t="s">
+      <c r="B19" s="3"/>
+      <c r="C19" s="3"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="3"/>
+    </row>
+    <row r="20" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="7" t="s">
+        <v>309</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>310</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>311</v>
+      </c>
+      <c r="D20" s="7"/>
+      <c r="E20" s="7"/>
+      <c r="F20" s="7"/>
+    </row>
+    <row r="21" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B21" s="4" t="s">
         <v>327</v>
       </c>
-      <c r="C15" s="4" t="s">
-        <v>300</v>
-      </c>
-      <c r="D15" s="4"/>
-      <c r="E15" s="4"/>
-      <c r="F15" s="4"/>
-    </row>
-    <row r="16" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="B16" s="8" t="s">
+      <c r="C21" s="4" t="s">
+        <v>313</v>
+      </c>
+      <c r="D21" s="4"/>
+      <c r="E21" s="4"/>
+      <c r="F21" s="4"/>
+    </row>
+    <row r="22" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="B22" s="8" t="s">
         <v>328</v>
       </c>
-      <c r="C16" s="8" t="s">
-        <v>329</v>
-      </c>
-      <c r="D16" s="8"/>
-      <c r="E16" s="8"/>
-      <c r="F16" s="8"/>
-    </row>
-    <row r="17" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>330</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>329</v>
-      </c>
-      <c r="D17" s="4"/>
-      <c r="E17" s="4"/>
-      <c r="F17" s="4"/>
-    </row>
-    <row r="18" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="B18" s="8" t="s">
-        <v>331</v>
-      </c>
-      <c r="C18" s="8" t="s">
-        <v>329</v>
-      </c>
-      <c r="D18" s="8"/>
-      <c r="E18" s="8"/>
-      <c r="F18" s="8"/>
-    </row>
-    <row r="19" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="B19" s="4" t="s">
-        <v>332</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>256</v>
-      </c>
-      <c r="D19" s="4"/>
-      <c r="E19" s="4"/>
-      <c r="F19" s="4"/>
-    </row>
-    <row r="21" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" s="3" t="s">
-        <v>333</v>
-      </c>
-      <c r="B21" s="3"/>
-      <c r="C21" s="3"/>
-      <c r="D21" s="3"/>
-      <c r="E21" s="3"/>
-      <c r="F21" s="3"/>
-      <c r="G21" s="3"/>
-    </row>
-    <row r="22" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" s="7" t="s">
-        <v>314</v>
-      </c>
-      <c r="B22" s="7" t="s">
-        <v>315</v>
-      </c>
-      <c r="C22" s="7" t="s">
-        <v>316</v>
-      </c>
-      <c r="D22" s="7"/>
-      <c r="E22" s="7"/>
-      <c r="F22" s="7"/>
+      <c r="C22" s="8" t="s">
+        <v>313</v>
+      </c>
+      <c r="D22" s="8"/>
+      <c r="E22" s="8"/>
+      <c r="F22" s="8"/>
     </row>
     <row r="23" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
         <v>91</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>334</v>
+        <v>329</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>300</v>
+        <v>313</v>
       </c>
       <c r="D23" s="4"/>
       <c r="E23" s="4"/>
@@ -4758,10 +4839,10 @@
         <v>91</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>335</v>
+        <v>330</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>300</v>
+        <v>256</v>
       </c>
       <c r="D24" s="8"/>
       <c r="E24" s="8"/>
@@ -4772,77 +4853,77 @@
         <v>91</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>336</v>
+        <v>331</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>300</v>
+        <v>313</v>
       </c>
       <c r="D25" s="4"/>
       <c r="E25" s="4"/>
       <c r="F25" s="4"/>
     </row>
-    <row r="26" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A26" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="B26" s="8" t="s">
-        <v>337</v>
-      </c>
-      <c r="C26" s="8" t="s">
-        <v>256</v>
-      </c>
-      <c r="D26" s="8"/>
-      <c r="E26" s="8"/>
-      <c r="F26" s="8"/>
-    </row>
-    <row r="27" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A27" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="B27" s="4" t="s">
-        <v>338</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>300</v>
-      </c>
-      <c r="D27" s="4"/>
-      <c r="E27" s="4"/>
-      <c r="F27" s="4"/>
-    </row>
-    <row r="29" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="3" t="s">
-        <v>339</v>
-      </c>
-      <c r="B29" s="3"/>
-      <c r="C29" s="3"/>
-      <c r="D29" s="3"/>
-      <c r="E29" s="3"/>
-      <c r="F29" s="3"/>
-      <c r="G29" s="3"/>
-    </row>
-    <row r="30" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A30" s="7" t="s">
-        <v>340</v>
-      </c>
-      <c r="B30" s="7" t="s">
-        <v>298</v>
-      </c>
-      <c r="C30" s="7" t="s">
-        <v>316</v>
-      </c>
-      <c r="D30" s="7"/>
-      <c r="E30" s="7"/>
-      <c r="F30" s="7"/>
+    <row r="27" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" s="3" t="s">
+        <v>332</v>
+      </c>
+      <c r="B27" s="3"/>
+      <c r="C27" s="3"/>
+      <c r="D27" s="3"/>
+      <c r="E27" s="3"/>
+      <c r="F27" s="3"/>
+      <c r="G27" s="3"/>
+    </row>
+    <row r="28" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" s="7" t="s">
+        <v>333</v>
+      </c>
+      <c r="B28" s="7" t="s">
+        <v>334</v>
+      </c>
+      <c r="C28" s="7" t="s">
+        <v>311</v>
+      </c>
+      <c r="D28" s="7"/>
+      <c r="E28" s="7"/>
+      <c r="F28" s="7"/>
+    </row>
+    <row r="29" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>335</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>323</v>
+      </c>
+      <c r="D29" s="4"/>
+      <c r="E29" s="4"/>
+      <c r="F29" s="4"/>
+    </row>
+    <row r="30" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="B30" s="8" t="s">
+        <v>336</v>
+      </c>
+      <c r="C30" s="8" t="s">
+        <v>313</v>
+      </c>
+      <c r="D30" s="8"/>
+      <c r="E30" s="8"/>
+      <c r="F30" s="8"/>
     </row>
     <row r="31" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
         <v>91</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>341</v>
+        <v>337</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>322</v>
+        <v>313</v>
       </c>
       <c r="D31" s="4"/>
       <c r="E31" s="4"/>
@@ -4853,10 +4934,10 @@
         <v>91</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>342</v>
+        <v>338</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>300</v>
+        <v>323</v>
       </c>
       <c r="D32" s="8"/>
       <c r="E32" s="8"/>
@@ -4867,10 +4948,10 @@
         <v>91</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>343</v>
+        <v>339</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>300</v>
+        <v>323</v>
       </c>
       <c r="D33" s="4"/>
       <c r="E33" s="4"/>
@@ -4881,59 +4962,17 @@
         <v>91</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>344</v>
+        <v>340</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>322</v>
+        <v>256</v>
       </c>
       <c r="D34" s="8"/>
       <c r="E34" s="8"/>
       <c r="F34" s="8"/>
     </row>
-    <row r="35" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A35" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="B35" s="4" t="s">
-        <v>345</v>
-      </c>
-      <c r="C35" s="4" t="s">
-        <v>322</v>
-      </c>
-      <c r="D35" s="4"/>
-      <c r="E35" s="4"/>
-      <c r="F35" s="4"/>
-    </row>
-    <row r="36" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A36" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="B36" s="8" t="s">
-        <v>346</v>
-      </c>
-      <c r="C36" s="8" t="s">
-        <v>256</v>
-      </c>
-      <c r="D36" s="8"/>
-      <c r="E36" s="8"/>
-      <c r="F36" s="8"/>
-    </row>
-    <row r="37" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A37" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="B37" s="4" t="s">
-        <v>347</v>
-      </c>
-      <c r="C37" s="4" t="s">
-        <v>300</v>
-      </c>
-      <c r="D37" s="4"/>
-      <c r="E37" s="4"/>
-      <c r="F37" s="4"/>
-    </row>
   </sheetData>
-  <mergeCells count="34">
+  <mergeCells count="31">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A3:G3"/>
@@ -4942,32 +4981,512 @@
     <mergeCell ref="C6:F6"/>
     <mergeCell ref="C7:F7"/>
     <mergeCell ref="C8:F8"/>
-    <mergeCell ref="C9:F9"/>
-    <mergeCell ref="A11:G11"/>
+    <mergeCell ref="A10:G10"/>
+    <mergeCell ref="C11:F11"/>
     <mergeCell ref="C12:F12"/>
     <mergeCell ref="C13:F13"/>
     <mergeCell ref="C14:F14"/>
     <mergeCell ref="C15:F15"/>
     <mergeCell ref="C16:F16"/>
     <mergeCell ref="C17:F17"/>
-    <mergeCell ref="C18:F18"/>
-    <mergeCell ref="C19:F19"/>
-    <mergeCell ref="A21:G21"/>
+    <mergeCell ref="A19:G19"/>
+    <mergeCell ref="C20:F20"/>
+    <mergeCell ref="C21:F21"/>
     <mergeCell ref="C22:F22"/>
     <mergeCell ref="C23:F23"/>
     <mergeCell ref="C24:F24"/>
     <mergeCell ref="C25:F25"/>
-    <mergeCell ref="C26:F26"/>
-    <mergeCell ref="C27:F27"/>
-    <mergeCell ref="A29:G29"/>
+    <mergeCell ref="A27:G27"/>
+    <mergeCell ref="C28:F28"/>
+    <mergeCell ref="C29:F29"/>
     <mergeCell ref="C30:F30"/>
     <mergeCell ref="C31:F31"/>
     <mergeCell ref="C32:F32"/>
     <mergeCell ref="C33:F33"/>
     <mergeCell ref="C34:F34"/>
-    <mergeCell ref="C35:F35"/>
-    <mergeCell ref="C36:F36"/>
-    <mergeCell ref="C37:F37"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G35"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="35" customWidth="1"/>
+    <col min="2" max="3" width="22" customWidth="1"/>
+    <col min="4" max="4" width="40" customWidth="1"/>
+    <col min="5" max="7" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="36" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>341</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+    </row>
+    <row r="2" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+    </row>
+    <row r="3" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="38" t="s">
+        <v>343</v>
+      </c>
+      <c r="B3" s="38"/>
+      <c r="C3" s="38"/>
+      <c r="D3" s="38"/>
+      <c r="E3" s="38"/>
+      <c r="F3" s="38"/>
+      <c r="G3" s="38"/>
+    </row>
+    <row r="5" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>344</v>
+      </c>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+    </row>
+    <row r="6" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
+        <v>345</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>346</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>347</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>348</v>
+      </c>
+      <c r="E6" s="7"/>
+      <c r="F6" s="7"/>
+      <c r="G6" s="7"/>
+    </row>
+    <row r="7" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="26" t="s">
+        <v>349</v>
+      </c>
+      <c r="B7" s="25" t="s">
+        <v>350</v>
+      </c>
+      <c r="C7" s="25" t="s">
+        <v>351</v>
+      </c>
+      <c r="D7" s="27" t="s">
+        <v>352</v>
+      </c>
+      <c r="E7" s="27"/>
+      <c r="F7" s="27"/>
+      <c r="G7" s="27"/>
+    </row>
+    <row r="8" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="30" t="s">
+        <v>353</v>
+      </c>
+      <c r="B8" s="29" t="s">
+        <v>354</v>
+      </c>
+      <c r="C8" s="29" t="s">
+        <v>355</v>
+      </c>
+      <c r="D8" s="31" t="s">
+        <v>356</v>
+      </c>
+      <c r="E8" s="31"/>
+      <c r="F8" s="31"/>
+      <c r="G8" s="31"/>
+    </row>
+    <row r="9" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="26" t="s">
+        <v>357</v>
+      </c>
+      <c r="B9" s="25" t="s">
+        <v>358</v>
+      </c>
+      <c r="C9" s="25" t="s">
+        <v>359</v>
+      </c>
+      <c r="D9" s="27" t="s">
+        <v>360</v>
+      </c>
+      <c r="E9" s="27"/>
+      <c r="F9" s="27"/>
+      <c r="G9" s="27"/>
+    </row>
+    <row r="10" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="30" t="s">
+        <v>361</v>
+      </c>
+      <c r="B10" s="29" t="s">
+        <v>351</v>
+      </c>
+      <c r="C10" s="29" t="s">
+        <v>362</v>
+      </c>
+      <c r="D10" s="31" t="s">
+        <v>363</v>
+      </c>
+      <c r="E10" s="31"/>
+      <c r="F10" s="31"/>
+      <c r="G10" s="31"/>
+    </row>
+    <row r="11" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="26" t="s">
+        <v>364</v>
+      </c>
+      <c r="B11" s="25" t="s">
+        <v>355</v>
+      </c>
+      <c r="C11" s="25" t="s">
+        <v>365</v>
+      </c>
+      <c r="D11" s="27" t="s">
+        <v>366</v>
+      </c>
+      <c r="E11" s="27"/>
+      <c r="F11" s="27"/>
+      <c r="G11" s="27"/>
+    </row>
+    <row r="12" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="30" t="s">
+        <v>367</v>
+      </c>
+      <c r="B12" s="29" t="s">
+        <v>358</v>
+      </c>
+      <c r="C12" s="29" t="s">
+        <v>368</v>
+      </c>
+      <c r="D12" s="31" t="s">
+        <v>369</v>
+      </c>
+      <c r="E12" s="31"/>
+      <c r="F12" s="31"/>
+      <c r="G12" s="31"/>
+    </row>
+    <row r="13" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="26" t="s">
+        <v>370</v>
+      </c>
+      <c r="B13" s="25" t="s">
+        <v>350</v>
+      </c>
+      <c r="C13" s="25" t="s">
+        <v>365</v>
+      </c>
+      <c r="D13" s="27" t="s">
+        <v>371</v>
+      </c>
+      <c r="E13" s="27"/>
+      <c r="F13" s="27"/>
+      <c r="G13" s="27"/>
+    </row>
+    <row r="14" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="30" t="s">
+        <v>372</v>
+      </c>
+      <c r="B14" s="29" t="s">
+        <v>354</v>
+      </c>
+      <c r="C14" s="29" t="s">
+        <v>355</v>
+      </c>
+      <c r="D14" s="31" t="s">
+        <v>373</v>
+      </c>
+      <c r="E14" s="31"/>
+      <c r="F14" s="31"/>
+      <c r="G14" s="31"/>
+    </row>
+    <row r="15" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="26" t="s">
+        <v>374</v>
+      </c>
+      <c r="B15" s="25" t="s">
+        <v>375</v>
+      </c>
+      <c r="C15" s="25" t="s">
+        <v>376</v>
+      </c>
+      <c r="D15" s="27" t="s">
+        <v>377</v>
+      </c>
+      <c r="E15" s="27"/>
+      <c r="F15" s="27"/>
+      <c r="G15" s="27"/>
+    </row>
+    <row r="17" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
+        <v>378</v>
+      </c>
+      <c r="B17" s="3"/>
+      <c r="C17" s="3"/>
+      <c r="D17" s="3"/>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
+      <c r="G17" s="3"/>
+    </row>
+    <row r="18" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>379</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>380</v>
+      </c>
+      <c r="D18" s="7"/>
+      <c r="E18" s="7"/>
+      <c r="F18" s="7"/>
+      <c r="G18" s="7"/>
+    </row>
+    <row r="19" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>381</v>
+      </c>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4"/>
+      <c r="F19" s="4"/>
+      <c r="G19" s="4"/>
+    </row>
+    <row r="20" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>382</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>383</v>
+      </c>
+      <c r="D20" s="8"/>
+      <c r="E20" s="8"/>
+      <c r="F20" s="8"/>
+      <c r="G20" s="8"/>
+    </row>
+    <row r="21" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>384</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>383</v>
+      </c>
+      <c r="D21" s="4"/>
+      <c r="E21" s="4"/>
+      <c r="F21" s="4"/>
+      <c r="G21" s="4"/>
+    </row>
+    <row r="22" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>385</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>381</v>
+      </c>
+      <c r="D22" s="8"/>
+      <c r="E22" s="8"/>
+      <c r="F22" s="8"/>
+      <c r="G22" s="8"/>
+    </row>
+    <row r="23" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>386</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>383</v>
+      </c>
+      <c r="D23" s="4"/>
+      <c r="E23" s="4"/>
+      <c r="F23" s="4"/>
+      <c r="G23" s="4"/>
+    </row>
+    <row r="24" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>387</v>
+      </c>
+      <c r="C24" s="8" t="s">
+        <v>388</v>
+      </c>
+      <c r="D24" s="8"/>
+      <c r="E24" s="8"/>
+      <c r="F24" s="8"/>
+      <c r="G24" s="8"/>
+    </row>
+    <row r="25" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>389</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>383</v>
+      </c>
+      <c r="D25" s="4"/>
+      <c r="E25" s="4"/>
+      <c r="F25" s="4"/>
+      <c r="G25" s="4"/>
+    </row>
+    <row r="27" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" s="39" t="s">
+        <v>390</v>
+      </c>
+      <c r="B27" s="39"/>
+      <c r="C27" s="39"/>
+      <c r="D27" s="39"/>
+      <c r="E27" s="39"/>
+      <c r="F27" s="39"/>
+      <c r="G27" s="39"/>
+    </row>
+    <row r="28" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" s="4" t="s">
+        <v>391</v>
+      </c>
+      <c r="B28" s="4"/>
+      <c r="C28" s="4"/>
+      <c r="D28" s="4"/>
+      <c r="E28" s="4"/>
+      <c r="F28" s="4"/>
+      <c r="G28" s="4"/>
+    </row>
+    <row r="29" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" s="15" t="s">
+        <v>392</v>
+      </c>
+      <c r="B29" s="15"/>
+      <c r="C29" s="15"/>
+      <c r="D29" s="15"/>
+      <c r="E29" s="15"/>
+      <c r="F29" s="15"/>
+      <c r="G29" s="15"/>
+    </row>
+    <row r="30" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" s="4" t="s">
+        <v>393</v>
+      </c>
+      <c r="B30" s="4"/>
+      <c r="C30" s="4"/>
+      <c r="D30" s="4"/>
+      <c r="E30" s="4"/>
+      <c r="F30" s="4"/>
+      <c r="G30" s="4"/>
+    </row>
+    <row r="31" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" s="15" t="s">
+        <v>394</v>
+      </c>
+      <c r="B31" s="15"/>
+      <c r="C31" s="15"/>
+      <c r="D31" s="15"/>
+      <c r="E31" s="15"/>
+      <c r="F31" s="15"/>
+      <c r="G31" s="15"/>
+    </row>
+    <row r="32" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" s="4" t="s">
+        <v>395</v>
+      </c>
+      <c r="B32" s="4"/>
+      <c r="C32" s="4"/>
+      <c r="D32" s="4"/>
+      <c r="E32" s="4"/>
+      <c r="F32" s="4"/>
+      <c r="G32" s="4"/>
+    </row>
+    <row r="34" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="B34" s="3"/>
+      <c r="C34" s="3"/>
+      <c r="D34" s="3"/>
+      <c r="E34" s="3"/>
+      <c r="F34" s="3"/>
+      <c r="G34" s="3"/>
+    </row>
+    <row r="35" ht="40" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" s="40" t="s">
+        <v>397</v>
+      </c>
+      <c r="B35" s="40"/>
+      <c r="C35" s="40"/>
+      <c r="D35" s="40"/>
+      <c r="E35" s="40"/>
+      <c r="F35" s="40"/>
+      <c r="G35" s="40"/>
+    </row>
+  </sheetData>
+  <mergeCells count="31">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A5:G5"/>
+    <mergeCell ref="D6:G6"/>
+    <mergeCell ref="D7:G7"/>
+    <mergeCell ref="D8:G8"/>
+    <mergeCell ref="D9:G9"/>
+    <mergeCell ref="D10:G10"/>
+    <mergeCell ref="D11:G11"/>
+    <mergeCell ref="D12:G12"/>
+    <mergeCell ref="D13:G13"/>
+    <mergeCell ref="D14:G14"/>
+    <mergeCell ref="D15:G15"/>
+    <mergeCell ref="A17:G17"/>
+    <mergeCell ref="C18:G18"/>
+    <mergeCell ref="C19:G19"/>
+    <mergeCell ref="C20:G20"/>
+    <mergeCell ref="C21:G21"/>
+    <mergeCell ref="C22:G22"/>
+    <mergeCell ref="C23:G23"/>
+    <mergeCell ref="C24:G24"/>
+    <mergeCell ref="C25:G25"/>
+    <mergeCell ref="A27:G27"/>
+    <mergeCell ref="A28:G28"/>
+    <mergeCell ref="A29:G29"/>
+    <mergeCell ref="A30:G30"/>
+    <mergeCell ref="A31:G31"/>
+    <mergeCell ref="A32:G32"/>
+    <mergeCell ref="A34:G34"/>
+    <mergeCell ref="A35:G35"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>